<commit_message>
BRME-4862: use valid restricted-picklist country code in test file
Country-code fields (Mobile/Business/Additional Phone Country Code) are restricted picklists; value '1' caused 'bad value for restricted picklist field: 1' errors on Map Columns. Generator now uses valid entry 'United States(+1)'; a blank cell still triggers the no-country-code error. Regenerated BRME-4862-mixed-errors-200rows.xlsx (same 50/25/25/25/25/25/25 distribution, verified).
</commit_message>
<xml_diff>
--- a/BRME-4862/test-data/BRME-4862-mixed-errors-200rows.xlsx
+++ b/BRME-4862/test-data/BRME-4862-mixed-errors-200rows.xlsx
@@ -484,19 +484,19 @@
         <v>2125550100</v>
       </c>
       <c r="J2" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K2" t="str">
         <v>9175550100</v>
       </c>
       <c r="L2" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M2" t="str">
         <v>6465550100</v>
       </c>
       <c r="N2" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -540,19 +540,19 @@
         <v>2125550100</v>
       </c>
       <c r="J3" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K3" t="str">
         <v>9175550100</v>
       </c>
       <c r="L3" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M3" t="str">
         <v>6465550100</v>
       </c>
       <c r="N3" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -596,19 +596,19 @@
         <v>2125550100</v>
       </c>
       <c r="J4" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K4" t="str">
         <v>9175550100</v>
       </c>
       <c r="L4" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M4" t="str">
         <v>6465550100</v>
       </c>
       <c r="N4" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -652,19 +652,19 @@
         <v>2125550100</v>
       </c>
       <c r="J5" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K5" t="str">
         <v>9175550100</v>
       </c>
       <c r="L5" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M5" t="str">
         <v>6465550100</v>
       </c>
       <c r="N5" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -708,19 +708,19 @@
         <v>2125550100</v>
       </c>
       <c r="J6" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K6" t="str">
         <v>9175550100</v>
       </c>
       <c r="L6" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M6" t="str">
         <v>6465550100</v>
       </c>
       <c r="N6" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -764,19 +764,19 @@
         <v>2125550100</v>
       </c>
       <c r="J7" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K7" t="str">
         <v>9175550100</v>
       </c>
       <c r="L7" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M7" t="str">
         <v>6465550100</v>
       </c>
       <c r="N7" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O7" t="str">
         <v/>
@@ -820,19 +820,19 @@
         <v>2125550100</v>
       </c>
       <c r="J8" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K8" t="str">
         <v>9175550100</v>
       </c>
       <c r="L8" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M8" t="str">
         <v>6465550100</v>
       </c>
       <c r="N8" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -876,19 +876,19 @@
         <v>2125550100</v>
       </c>
       <c r="J9" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K9" t="str">
         <v>9175550100</v>
       </c>
       <c r="L9" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M9" t="str">
         <v>6465550100</v>
       </c>
       <c r="N9" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -932,19 +932,19 @@
         <v>2125550100</v>
       </c>
       <c r="J10" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K10" t="str">
         <v>9175550100</v>
       </c>
       <c r="L10" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M10" t="str">
         <v>6465550100</v>
       </c>
       <c r="N10" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -988,19 +988,19 @@
         <v>2125550100</v>
       </c>
       <c r="J11" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K11" t="str">
         <v>9175550100</v>
       </c>
       <c r="L11" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M11" t="str">
         <v>6465550100</v>
       </c>
       <c r="N11" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1044,19 +1044,19 @@
         <v>2125550100</v>
       </c>
       <c r="J12" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K12" t="str">
         <v>9175550100</v>
       </c>
       <c r="L12" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M12" t="str">
         <v>6465550100</v>
       </c>
       <c r="N12" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1100,19 +1100,19 @@
         <v>2125550100</v>
       </c>
       <c r="J13" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K13" t="str">
         <v>9175550100</v>
       </c>
       <c r="L13" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M13" t="str">
         <v>6465550100</v>
       </c>
       <c r="N13" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O13" t="str">
         <v/>
@@ -1156,19 +1156,19 @@
         <v>2125550100</v>
       </c>
       <c r="J14" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K14" t="str">
         <v>9175550100</v>
       </c>
       <c r="L14" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M14" t="str">
         <v>6465550100</v>
       </c>
       <c r="N14" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O14" t="str">
         <v/>
@@ -1212,19 +1212,19 @@
         <v>2125550100</v>
       </c>
       <c r="J15" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K15" t="str">
         <v>9175550100</v>
       </c>
       <c r="L15" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M15" t="str">
         <v>6465550100</v>
       </c>
       <c r="N15" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -1268,19 +1268,19 @@
         <v>2125550100</v>
       </c>
       <c r="J16" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K16" t="str">
         <v>9175550100</v>
       </c>
       <c r="L16" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M16" t="str">
         <v>6465550100</v>
       </c>
       <c r="N16" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O16" t="str">
         <v/>
@@ -1324,19 +1324,19 @@
         <v>2125550100</v>
       </c>
       <c r="J17" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K17" t="str">
         <v>9175550100</v>
       </c>
       <c r="L17" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M17" t="str">
         <v>6465550100</v>
       </c>
       <c r="N17" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O17" t="str">
         <v/>
@@ -1380,19 +1380,19 @@
         <v>2125550100</v>
       </c>
       <c r="J18" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K18" t="str">
         <v>9175550100</v>
       </c>
       <c r="L18" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M18" t="str">
         <v>6465550100</v>
       </c>
       <c r="N18" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O18" t="str">
         <v/>
@@ -1436,19 +1436,19 @@
         <v>2125550100</v>
       </c>
       <c r="J19" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K19" t="str">
         <v>9175550100</v>
       </c>
       <c r="L19" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M19" t="str">
         <v>6465550100</v>
       </c>
       <c r="N19" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O19" t="str">
         <v/>
@@ -1492,19 +1492,19 @@
         <v>2125550100</v>
       </c>
       <c r="J20" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K20" t="str">
         <v>9175550100</v>
       </c>
       <c r="L20" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M20" t="str">
         <v>6465550100</v>
       </c>
       <c r="N20" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O20" t="str">
         <v/>
@@ -1548,19 +1548,19 @@
         <v>2125550100</v>
       </c>
       <c r="J21" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K21" t="str">
         <v>9175550100</v>
       </c>
       <c r="L21" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M21" t="str">
         <v>6465550100</v>
       </c>
       <c r="N21" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O21" t="str">
         <v/>
@@ -1604,19 +1604,19 @@
         <v>2125550100</v>
       </c>
       <c r="J22" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K22" t="str">
         <v>9175550100</v>
       </c>
       <c r="L22" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M22" t="str">
         <v>6465550100</v>
       </c>
       <c r="N22" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O22" t="str">
         <v/>
@@ -1660,19 +1660,19 @@
         <v>2125550100</v>
       </c>
       <c r="J23" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K23" t="str">
         <v>9175550100</v>
       </c>
       <c r="L23" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M23" t="str">
         <v>6465550100</v>
       </c>
       <c r="N23" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O23" t="str">
         <v/>
@@ -1716,19 +1716,19 @@
         <v>2125550100</v>
       </c>
       <c r="J24" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K24" t="str">
         <v>9175550100</v>
       </c>
       <c r="L24" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M24" t="str">
         <v>6465550100</v>
       </c>
       <c r="N24" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O24" t="str">
         <v/>
@@ -1772,19 +1772,19 @@
         <v>2125550100</v>
       </c>
       <c r="J25" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K25" t="str">
         <v>9175550100</v>
       </c>
       <c r="L25" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M25" t="str">
         <v>6465550100</v>
       </c>
       <c r="N25" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O25" t="str">
         <v/>
@@ -1828,19 +1828,19 @@
         <v>2125550100</v>
       </c>
       <c r="J26" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K26" t="str">
         <v>9175550100</v>
       </c>
       <c r="L26" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M26" t="str">
         <v>6465550100</v>
       </c>
       <c r="N26" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O26" t="str">
         <v/>
@@ -1884,19 +1884,19 @@
         <v>2125550100</v>
       </c>
       <c r="J27" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K27" t="str">
         <v>9175550100</v>
       </c>
       <c r="L27" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M27" t="str">
         <v>6465550100</v>
       </c>
       <c r="N27" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O27" t="str">
         <v/>
@@ -1940,19 +1940,19 @@
         <v>2125550100</v>
       </c>
       <c r="J28" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K28" t="str">
         <v>9175550100</v>
       </c>
       <c r="L28" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M28" t="str">
         <v>6465550100</v>
       </c>
       <c r="N28" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -1996,19 +1996,19 @@
         <v>2125550100</v>
       </c>
       <c r="J29" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K29" t="str">
         <v>9175550100</v>
       </c>
       <c r="L29" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M29" t="str">
         <v>6465550100</v>
       </c>
       <c r="N29" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O29" t="str">
         <v/>
@@ -2052,19 +2052,19 @@
         <v>2125550100</v>
       </c>
       <c r="J30" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K30" t="str">
         <v>9175550100</v>
       </c>
       <c r="L30" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M30" t="str">
         <v>6465550100</v>
       </c>
       <c r="N30" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O30" t="str">
         <v/>
@@ -2108,19 +2108,19 @@
         <v>2125550100</v>
       </c>
       <c r="J31" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K31" t="str">
         <v>9175550100</v>
       </c>
       <c r="L31" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M31" t="str">
         <v>6465550100</v>
       </c>
       <c r="N31" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O31" t="str">
         <v/>
@@ -2164,19 +2164,19 @@
         <v>2125550100</v>
       </c>
       <c r="J32" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K32" t="str">
         <v>9175550100</v>
       </c>
       <c r="L32" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M32" t="str">
         <v>6465550100</v>
       </c>
       <c r="N32" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O32" t="str">
         <v/>
@@ -2220,19 +2220,19 @@
         <v>2125550100</v>
       </c>
       <c r="J33" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K33" t="str">
         <v>9175550100</v>
       </c>
       <c r="L33" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M33" t="str">
         <v>6465550100</v>
       </c>
       <c r="N33" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O33" t="str">
         <v/>
@@ -2276,19 +2276,19 @@
         <v>2125550100</v>
       </c>
       <c r="J34" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K34" t="str">
         <v>9175550100</v>
       </c>
       <c r="L34" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M34" t="str">
         <v>6465550100</v>
       </c>
       <c r="N34" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O34" t="str">
         <v/>
@@ -2332,19 +2332,19 @@
         <v>2125550100</v>
       </c>
       <c r="J35" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K35" t="str">
         <v>9175550100</v>
       </c>
       <c r="L35" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M35" t="str">
         <v>6465550100</v>
       </c>
       <c r="N35" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O35" t="str">
         <v/>
@@ -2388,19 +2388,19 @@
         <v>2125550100</v>
       </c>
       <c r="J36" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K36" t="str">
         <v>9175550100</v>
       </c>
       <c r="L36" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M36" t="str">
         <v>6465550100</v>
       </c>
       <c r="N36" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O36" t="str">
         <v/>
@@ -2444,19 +2444,19 @@
         <v>2125550100</v>
       </c>
       <c r="J37" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K37" t="str">
         <v>9175550100</v>
       </c>
       <c r="L37" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M37" t="str">
         <v>6465550100</v>
       </c>
       <c r="N37" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O37" t="str">
         <v/>
@@ -2500,19 +2500,19 @@
         <v>2125550100</v>
       </c>
       <c r="J38" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K38" t="str">
         <v>9175550100</v>
       </c>
       <c r="L38" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M38" t="str">
         <v>6465550100</v>
       </c>
       <c r="N38" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O38" t="str">
         <v/>
@@ -2556,19 +2556,19 @@
         <v>2125550100</v>
       </c>
       <c r="J39" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K39" t="str">
         <v>9175550100</v>
       </c>
       <c r="L39" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M39" t="str">
         <v>6465550100</v>
       </c>
       <c r="N39" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O39" t="str">
         <v/>
@@ -2612,19 +2612,19 @@
         <v>2125550100</v>
       </c>
       <c r="J40" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K40" t="str">
         <v>9175550100</v>
       </c>
       <c r="L40" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M40" t="str">
         <v>6465550100</v>
       </c>
       <c r="N40" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O40" t="str">
         <v/>
@@ -2668,19 +2668,19 @@
         <v>2125550100</v>
       </c>
       <c r="J41" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K41" t="str">
         <v>9175550100</v>
       </c>
       <c r="L41" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M41" t="str">
         <v>6465550100</v>
       </c>
       <c r="N41" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O41" t="str">
         <v/>
@@ -2724,19 +2724,19 @@
         <v>2125550100</v>
       </c>
       <c r="J42" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K42" t="str">
         <v>9175550100</v>
       </c>
       <c r="L42" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M42" t="str">
         <v>6465550100</v>
       </c>
       <c r="N42" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O42" t="str">
         <v/>
@@ -2780,19 +2780,19 @@
         <v>2125550100</v>
       </c>
       <c r="J43" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K43" t="str">
         <v>9175550100</v>
       </c>
       <c r="L43" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M43" t="str">
         <v>6465550100</v>
       </c>
       <c r="N43" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O43" t="str">
         <v/>
@@ -2836,19 +2836,19 @@
         <v>2125550100</v>
       </c>
       <c r="J44" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K44" t="str">
         <v>9175550100</v>
       </c>
       <c r="L44" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M44" t="str">
         <v>6465550100</v>
       </c>
       <c r="N44" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O44" t="str">
         <v/>
@@ -2892,19 +2892,19 @@
         <v>2125550100</v>
       </c>
       <c r="J45" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K45" t="str">
         <v>9175550100</v>
       </c>
       <c r="L45" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M45" t="str">
         <v>6465550100</v>
       </c>
       <c r="N45" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -2948,19 +2948,19 @@
         <v>2125550100</v>
       </c>
       <c r="J46" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K46" t="str">
         <v>9175550100</v>
       </c>
       <c r="L46" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M46" t="str">
         <v>6465550100</v>
       </c>
       <c r="N46" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O46" t="str">
         <v/>
@@ -3004,19 +3004,19 @@
         <v>2125550100</v>
       </c>
       <c r="J47" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K47" t="str">
         <v>9175550100</v>
       </c>
       <c r="L47" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M47" t="str">
         <v>6465550100</v>
       </c>
       <c r="N47" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O47" t="str">
         <v/>
@@ -3060,19 +3060,19 @@
         <v>2125550100</v>
       </c>
       <c r="J48" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K48" t="str">
         <v>9175550100</v>
       </c>
       <c r="L48" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M48" t="str">
         <v>6465550100</v>
       </c>
       <c r="N48" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O48" t="str">
         <v/>
@@ -3116,19 +3116,19 @@
         <v>2125550100</v>
       </c>
       <c r="J49" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K49" t="str">
         <v>9175550100</v>
       </c>
       <c r="L49" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M49" t="str">
         <v>6465550100</v>
       </c>
       <c r="N49" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O49" t="str">
         <v/>
@@ -3172,19 +3172,19 @@
         <v>2125550100</v>
       </c>
       <c r="J50" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K50" t="str">
         <v>9175550100</v>
       </c>
       <c r="L50" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M50" t="str">
         <v>6465550100</v>
       </c>
       <c r="N50" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O50" t="str">
         <v/>
@@ -3228,19 +3228,19 @@
         <v>2125550100</v>
       </c>
       <c r="J51" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K51" t="str">
         <v>9175550100</v>
       </c>
       <c r="L51" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M51" t="str">
         <v>6465550100</v>
       </c>
       <c r="N51" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O51" t="str">
         <v/>
@@ -3284,7 +3284,7 @@
         <v>2125550100</v>
       </c>
       <c r="J52" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K52" t="str">
         <v>9175550100</v>
@@ -3296,7 +3296,7 @@
         <v>6465550100</v>
       </c>
       <c r="N52" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O52" t="str">
         <v/>
@@ -3340,7 +3340,7 @@
         <v>2125550100</v>
       </c>
       <c r="J53" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K53" t="str">
         <v>9175550100</v>
@@ -3352,7 +3352,7 @@
         <v>6465550100</v>
       </c>
       <c r="N53" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O53" t="str">
         <v/>
@@ -3396,7 +3396,7 @@
         <v>2125550100</v>
       </c>
       <c r="J54" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K54" t="str">
         <v>9175550100</v>
@@ -3408,7 +3408,7 @@
         <v>6465550100</v>
       </c>
       <c r="N54" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O54" t="str">
         <v/>
@@ -3452,7 +3452,7 @@
         <v>2125550100</v>
       </c>
       <c r="J55" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K55" t="str">
         <v>9175550100</v>
@@ -3464,7 +3464,7 @@
         <v>6465550100</v>
       </c>
       <c r="N55" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O55" t="str">
         <v/>
@@ -3508,7 +3508,7 @@
         <v>2125550100</v>
       </c>
       <c r="J56" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K56" t="str">
         <v>9175550100</v>
@@ -3520,7 +3520,7 @@
         <v>6465550100</v>
       </c>
       <c r="N56" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O56" t="str">
         <v/>
@@ -3564,7 +3564,7 @@
         <v>2125550100</v>
       </c>
       <c r="J57" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K57" t="str">
         <v>9175550100</v>
@@ -3576,7 +3576,7 @@
         <v>6465550100</v>
       </c>
       <c r="N57" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O57" t="str">
         <v/>
@@ -3620,7 +3620,7 @@
         <v>2125550100</v>
       </c>
       <c r="J58" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K58" t="str">
         <v>9175550100</v>
@@ -3632,7 +3632,7 @@
         <v>6465550100</v>
       </c>
       <c r="N58" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O58" t="str">
         <v/>
@@ -3676,7 +3676,7 @@
         <v>2125550100</v>
       </c>
       <c r="J59" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K59" t="str">
         <v>9175550100</v>
@@ -3688,7 +3688,7 @@
         <v>6465550100</v>
       </c>
       <c r="N59" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O59" t="str">
         <v/>
@@ -3732,7 +3732,7 @@
         <v>2125550100</v>
       </c>
       <c r="J60" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K60" t="str">
         <v>9175550100</v>
@@ -3744,7 +3744,7 @@
         <v>6465550100</v>
       </c>
       <c r="N60" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O60" t="str">
         <v/>
@@ -3788,7 +3788,7 @@
         <v>2125550100</v>
       </c>
       <c r="J61" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K61" t="str">
         <v>9175550100</v>
@@ -3800,7 +3800,7 @@
         <v>6465550100</v>
       </c>
       <c r="N61" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O61" t="str">
         <v/>
@@ -3844,7 +3844,7 @@
         <v>2125550100</v>
       </c>
       <c r="J62" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K62" t="str">
         <v>9175550100</v>
@@ -3856,7 +3856,7 @@
         <v>6465550100</v>
       </c>
       <c r="N62" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O62" t="str">
         <v/>
@@ -3900,7 +3900,7 @@
         <v>2125550100</v>
       </c>
       <c r="J63" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K63" t="str">
         <v>9175550100</v>
@@ -3912,7 +3912,7 @@
         <v>6465550100</v>
       </c>
       <c r="N63" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O63" t="str">
         <v/>
@@ -3956,7 +3956,7 @@
         <v>2125550100</v>
       </c>
       <c r="J64" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K64" t="str">
         <v>9175550100</v>
@@ -3968,7 +3968,7 @@
         <v>6465550100</v>
       </c>
       <c r="N64" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O64" t="str">
         <v/>
@@ -4012,7 +4012,7 @@
         <v>2125550100</v>
       </c>
       <c r="J65" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K65" t="str">
         <v>9175550100</v>
@@ -4024,7 +4024,7 @@
         <v>6465550100</v>
       </c>
       <c r="N65" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O65" t="str">
         <v/>
@@ -4068,7 +4068,7 @@
         <v>2125550100</v>
       </c>
       <c r="J66" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K66" t="str">
         <v>9175550100</v>
@@ -4080,7 +4080,7 @@
         <v>6465550100</v>
       </c>
       <c r="N66" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O66" t="str">
         <v/>
@@ -4124,7 +4124,7 @@
         <v>2125550100</v>
       </c>
       <c r="J67" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K67" t="str">
         <v>9175550100</v>
@@ -4136,7 +4136,7 @@
         <v>6465550100</v>
       </c>
       <c r="N67" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O67" t="str">
         <v/>
@@ -4180,7 +4180,7 @@
         <v>2125550100</v>
       </c>
       <c r="J68" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K68" t="str">
         <v>9175550100</v>
@@ -4192,7 +4192,7 @@
         <v>6465550100</v>
       </c>
       <c r="N68" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O68" t="str">
         <v/>
@@ -4236,7 +4236,7 @@
         <v>2125550100</v>
       </c>
       <c r="J69" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K69" t="str">
         <v>9175550100</v>
@@ -4248,7 +4248,7 @@
         <v>6465550100</v>
       </c>
       <c r="N69" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O69" t="str">
         <v/>
@@ -4292,7 +4292,7 @@
         <v>2125550100</v>
       </c>
       <c r="J70" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K70" t="str">
         <v>9175550100</v>
@@ -4304,7 +4304,7 @@
         <v>6465550100</v>
       </c>
       <c r="N70" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O70" t="str">
         <v/>
@@ -4348,7 +4348,7 @@
         <v>2125550100</v>
       </c>
       <c r="J71" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K71" t="str">
         <v>9175550100</v>
@@ -4360,7 +4360,7 @@
         <v>6465550100</v>
       </c>
       <c r="N71" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O71" t="str">
         <v/>
@@ -4404,7 +4404,7 @@
         <v>2125550100</v>
       </c>
       <c r="J72" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K72" t="str">
         <v>9175550100</v>
@@ -4416,7 +4416,7 @@
         <v>6465550100</v>
       </c>
       <c r="N72" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O72" t="str">
         <v/>
@@ -4460,7 +4460,7 @@
         <v>2125550100</v>
       </c>
       <c r="J73" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K73" t="str">
         <v>9175550100</v>
@@ -4472,7 +4472,7 @@
         <v>6465550100</v>
       </c>
       <c r="N73" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O73" t="str">
         <v/>
@@ -4516,7 +4516,7 @@
         <v>2125550100</v>
       </c>
       <c r="J74" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K74" t="str">
         <v>9175550100</v>
@@ -4528,7 +4528,7 @@
         <v>6465550100</v>
       </c>
       <c r="N74" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O74" t="str">
         <v/>
@@ -4572,7 +4572,7 @@
         <v>2125550100</v>
       </c>
       <c r="J75" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K75" t="str">
         <v>9175550100</v>
@@ -4584,7 +4584,7 @@
         <v>6465550100</v>
       </c>
       <c r="N75" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O75" t="str">
         <v/>
@@ -4628,7 +4628,7 @@
         <v>2125550100</v>
       </c>
       <c r="J76" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K76" t="str">
         <v>9175550100</v>
@@ -4640,7 +4640,7 @@
         <v>6465550100</v>
       </c>
       <c r="N76" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O76" t="str">
         <v/>
@@ -4690,13 +4690,13 @@
         <v>9175550100</v>
       </c>
       <c r="L77" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M77" t="str">
         <v>6465550100</v>
       </c>
       <c r="N77" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O77" t="str">
         <v/>
@@ -4746,13 +4746,13 @@
         <v>9175550100</v>
       </c>
       <c r="L78" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M78" t="str">
         <v>6465550100</v>
       </c>
       <c r="N78" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O78" t="str">
         <v/>
@@ -4802,13 +4802,13 @@
         <v>9175550100</v>
       </c>
       <c r="L79" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M79" t="str">
         <v>6465550100</v>
       </c>
       <c r="N79" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O79" t="str">
         <v/>
@@ -4858,13 +4858,13 @@
         <v>9175550100</v>
       </c>
       <c r="L80" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M80" t="str">
         <v>6465550100</v>
       </c>
       <c r="N80" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O80" t="str">
         <v/>
@@ -4914,13 +4914,13 @@
         <v>9175550100</v>
       </c>
       <c r="L81" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M81" t="str">
         <v>6465550100</v>
       </c>
       <c r="N81" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O81" t="str">
         <v/>
@@ -4970,13 +4970,13 @@
         <v>9175550100</v>
       </c>
       <c r="L82" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M82" t="str">
         <v>6465550100</v>
       </c>
       <c r="N82" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O82" t="str">
         <v/>
@@ -5026,13 +5026,13 @@
         <v>9175550100</v>
       </c>
       <c r="L83" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M83" t="str">
         <v>6465550100</v>
       </c>
       <c r="N83" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O83" t="str">
         <v/>
@@ -5082,13 +5082,13 @@
         <v>9175550100</v>
       </c>
       <c r="L84" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M84" t="str">
         <v>6465550100</v>
       </c>
       <c r="N84" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O84" t="str">
         <v/>
@@ -5138,13 +5138,13 @@
         <v>9175550100</v>
       </c>
       <c r="L85" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M85" t="str">
         <v>6465550100</v>
       </c>
       <c r="N85" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O85" t="str">
         <v/>
@@ -5194,13 +5194,13 @@
         <v>9175550100</v>
       </c>
       <c r="L86" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M86" t="str">
         <v>6465550100</v>
       </c>
       <c r="N86" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O86" t="str">
         <v/>
@@ -5250,13 +5250,13 @@
         <v>9175550100</v>
       </c>
       <c r="L87" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M87" t="str">
         <v>6465550100</v>
       </c>
       <c r="N87" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O87" t="str">
         <v/>
@@ -5306,13 +5306,13 @@
         <v>9175550100</v>
       </c>
       <c r="L88" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M88" t="str">
         <v>6465550100</v>
       </c>
       <c r="N88" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O88" t="str">
         <v/>
@@ -5362,13 +5362,13 @@
         <v>9175550100</v>
       </c>
       <c r="L89" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M89" t="str">
         <v>6465550100</v>
       </c>
       <c r="N89" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O89" t="str">
         <v/>
@@ -5418,13 +5418,13 @@
         <v>9175550100</v>
       </c>
       <c r="L90" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M90" t="str">
         <v>6465550100</v>
       </c>
       <c r="N90" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O90" t="str">
         <v/>
@@ -5474,13 +5474,13 @@
         <v>9175550100</v>
       </c>
       <c r="L91" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M91" t="str">
         <v>6465550100</v>
       </c>
       <c r="N91" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O91" t="str">
         <v/>
@@ -5530,13 +5530,13 @@
         <v>9175550100</v>
       </c>
       <c r="L92" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M92" t="str">
         <v>6465550100</v>
       </c>
       <c r="N92" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O92" t="str">
         <v/>
@@ -5586,13 +5586,13 @@
         <v>9175550100</v>
       </c>
       <c r="L93" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M93" t="str">
         <v>6465550100</v>
       </c>
       <c r="N93" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O93" t="str">
         <v/>
@@ -5642,13 +5642,13 @@
         <v>9175550100</v>
       </c>
       <c r="L94" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M94" t="str">
         <v>6465550100</v>
       </c>
       <c r="N94" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O94" t="str">
         <v/>
@@ -5698,13 +5698,13 @@
         <v>9175550100</v>
       </c>
       <c r="L95" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M95" t="str">
         <v>6465550100</v>
       </c>
       <c r="N95" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O95" t="str">
         <v/>
@@ -5754,13 +5754,13 @@
         <v>9175550100</v>
       </c>
       <c r="L96" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M96" t="str">
         <v>6465550100</v>
       </c>
       <c r="N96" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O96" t="str">
         <v/>
@@ -5810,13 +5810,13 @@
         <v>9175550100</v>
       </c>
       <c r="L97" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M97" t="str">
         <v>6465550100</v>
       </c>
       <c r="N97" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O97" t="str">
         <v/>
@@ -5866,13 +5866,13 @@
         <v>9175550100</v>
       </c>
       <c r="L98" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M98" t="str">
         <v>6465550100</v>
       </c>
       <c r="N98" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O98" t="str">
         <v/>
@@ -5922,13 +5922,13 @@
         <v>9175550100</v>
       </c>
       <c r="L99" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M99" t="str">
         <v>6465550100</v>
       </c>
       <c r="N99" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O99" t="str">
         <v/>
@@ -5978,13 +5978,13 @@
         <v>9175550100</v>
       </c>
       <c r="L100" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M100" t="str">
         <v>6465550100</v>
       </c>
       <c r="N100" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O100" t="str">
         <v/>
@@ -6034,13 +6034,13 @@
         <v>9175550100</v>
       </c>
       <c r="L101" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M101" t="str">
         <v>6465550100</v>
       </c>
       <c r="N101" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O101" t="str">
         <v/>
@@ -6084,13 +6084,13 @@
         <v>2125550100</v>
       </c>
       <c r="J102" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K102" t="str">
         <v>9175550100</v>
       </c>
       <c r="L102" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M102" t="str">
         <v>6465550100</v>
@@ -6140,13 +6140,13 @@
         <v>2125550100</v>
       </c>
       <c r="J103" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K103" t="str">
         <v>9175550100</v>
       </c>
       <c r="L103" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M103" t="str">
         <v>6465550100</v>
@@ -6196,13 +6196,13 @@
         <v>2125550100</v>
       </c>
       <c r="J104" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K104" t="str">
         <v>9175550100</v>
       </c>
       <c r="L104" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M104" t="str">
         <v>6465550100</v>
@@ -6252,13 +6252,13 @@
         <v>2125550100</v>
       </c>
       <c r="J105" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K105" t="str">
         <v>9175550100</v>
       </c>
       <c r="L105" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M105" t="str">
         <v>6465550100</v>
@@ -6308,13 +6308,13 @@
         <v>2125550100</v>
       </c>
       <c r="J106" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K106" t="str">
         <v>9175550100</v>
       </c>
       <c r="L106" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M106" t="str">
         <v>6465550100</v>
@@ -6364,13 +6364,13 @@
         <v>2125550100</v>
       </c>
       <c r="J107" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K107" t="str">
         <v>9175550100</v>
       </c>
       <c r="L107" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M107" t="str">
         <v>6465550100</v>
@@ -6420,13 +6420,13 @@
         <v>2125550100</v>
       </c>
       <c r="J108" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K108" t="str">
         <v>9175550100</v>
       </c>
       <c r="L108" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M108" t="str">
         <v>6465550100</v>
@@ -6476,13 +6476,13 @@
         <v>2125550100</v>
       </c>
       <c r="J109" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K109" t="str">
         <v>9175550100</v>
       </c>
       <c r="L109" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M109" t="str">
         <v>6465550100</v>
@@ -6532,13 +6532,13 @@
         <v>2125550100</v>
       </c>
       <c r="J110" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K110" t="str">
         <v>9175550100</v>
       </c>
       <c r="L110" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M110" t="str">
         <v>6465550100</v>
@@ -6588,13 +6588,13 @@
         <v>2125550100</v>
       </c>
       <c r="J111" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K111" t="str">
         <v>9175550100</v>
       </c>
       <c r="L111" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M111" t="str">
         <v>6465550100</v>
@@ -6644,13 +6644,13 @@
         <v>2125550100</v>
       </c>
       <c r="J112" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K112" t="str">
         <v>9175550100</v>
       </c>
       <c r="L112" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M112" t="str">
         <v>6465550100</v>
@@ -6700,13 +6700,13 @@
         <v>2125550100</v>
       </c>
       <c r="J113" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K113" t="str">
         <v>9175550100</v>
       </c>
       <c r="L113" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M113" t="str">
         <v>6465550100</v>
@@ -6756,13 +6756,13 @@
         <v>2125550100</v>
       </c>
       <c r="J114" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K114" t="str">
         <v>9175550100</v>
       </c>
       <c r="L114" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M114" t="str">
         <v>6465550100</v>
@@ -6812,13 +6812,13 @@
         <v>2125550100</v>
       </c>
       <c r="J115" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K115" t="str">
         <v>9175550100</v>
       </c>
       <c r="L115" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M115" t="str">
         <v>6465550100</v>
@@ -6868,13 +6868,13 @@
         <v>2125550100</v>
       </c>
       <c r="J116" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K116" t="str">
         <v>9175550100</v>
       </c>
       <c r="L116" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M116" t="str">
         <v>6465550100</v>
@@ -6924,13 +6924,13 @@
         <v>2125550100</v>
       </c>
       <c r="J117" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K117" t="str">
         <v>9175550100</v>
       </c>
       <c r="L117" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M117" t="str">
         <v>6465550100</v>
@@ -6980,13 +6980,13 @@
         <v>2125550100</v>
       </c>
       <c r="J118" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K118" t="str">
         <v>9175550100</v>
       </c>
       <c r="L118" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M118" t="str">
         <v>6465550100</v>
@@ -7036,13 +7036,13 @@
         <v>2125550100</v>
       </c>
       <c r="J119" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K119" t="str">
         <v>9175550100</v>
       </c>
       <c r="L119" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M119" t="str">
         <v>6465550100</v>
@@ -7092,13 +7092,13 @@
         <v>2125550100</v>
       </c>
       <c r="J120" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K120" t="str">
         <v>9175550100</v>
       </c>
       <c r="L120" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M120" t="str">
         <v>6465550100</v>
@@ -7148,13 +7148,13 @@
         <v>2125550100</v>
       </c>
       <c r="J121" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K121" t="str">
         <v>9175550100</v>
       </c>
       <c r="L121" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M121" t="str">
         <v>6465550100</v>
@@ -7204,13 +7204,13 @@
         <v>2125550100</v>
       </c>
       <c r="J122" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K122" t="str">
         <v>9175550100</v>
       </c>
       <c r="L122" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M122" t="str">
         <v>6465550100</v>
@@ -7260,13 +7260,13 @@
         <v>2125550100</v>
       </c>
       <c r="J123" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K123" t="str">
         <v>9175550100</v>
       </c>
       <c r="L123" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M123" t="str">
         <v>6465550100</v>
@@ -7316,13 +7316,13 @@
         <v>2125550100</v>
       </c>
       <c r="J124" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K124" t="str">
         <v>9175550100</v>
       </c>
       <c r="L124" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M124" t="str">
         <v>6465550100</v>
@@ -7372,13 +7372,13 @@
         <v>2125550100</v>
       </c>
       <c r="J125" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K125" t="str">
         <v>9175550100</v>
       </c>
       <c r="L125" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M125" t="str">
         <v>6465550100</v>
@@ -7428,13 +7428,13 @@
         <v>2125550100</v>
       </c>
       <c r="J126" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K126" t="str">
         <v>9175550100</v>
       </c>
       <c r="L126" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M126" t="str">
         <v>6465550100</v>
@@ -7484,19 +7484,19 @@
         <v>2125550100</v>
       </c>
       <c r="J127" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K127" t="str">
         <v>9175550100</v>
       </c>
       <c r="L127" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M127" t="str">
         <v>6465550100</v>
       </c>
       <c r="N127" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O127" t="str">
         <v/>
@@ -7540,19 +7540,19 @@
         <v>2125550100</v>
       </c>
       <c r="J128" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K128" t="str">
         <v>9175550100</v>
       </c>
       <c r="L128" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M128" t="str">
         <v>6465550100</v>
       </c>
       <c r="N128" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O128" t="str">
         <v/>
@@ -7596,19 +7596,19 @@
         <v>2125550100</v>
       </c>
       <c r="J129" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K129" t="str">
         <v>9175550100</v>
       </c>
       <c r="L129" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M129" t="str">
         <v>6465550100</v>
       </c>
       <c r="N129" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O129" t="str">
         <v/>
@@ -7652,19 +7652,19 @@
         <v>2125550100</v>
       </c>
       <c r="J130" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K130" t="str">
         <v>9175550100</v>
       </c>
       <c r="L130" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M130" t="str">
         <v>6465550100</v>
       </c>
       <c r="N130" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O130" t="str">
         <v/>
@@ -7708,19 +7708,19 @@
         <v>2125550100</v>
       </c>
       <c r="J131" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K131" t="str">
         <v>9175550100</v>
       </c>
       <c r="L131" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M131" t="str">
         <v>6465550100</v>
       </c>
       <c r="N131" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O131" t="str">
         <v/>
@@ -7764,19 +7764,19 @@
         <v>2125550100</v>
       </c>
       <c r="J132" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K132" t="str">
         <v>9175550100</v>
       </c>
       <c r="L132" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M132" t="str">
         <v>6465550100</v>
       </c>
       <c r="N132" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O132" t="str">
         <v/>
@@ -7820,19 +7820,19 @@
         <v>2125550100</v>
       </c>
       <c r="J133" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K133" t="str">
         <v>9175550100</v>
       </c>
       <c r="L133" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M133" t="str">
         <v>6465550100</v>
       </c>
       <c r="N133" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O133" t="str">
         <v/>
@@ -7876,19 +7876,19 @@
         <v>2125550100</v>
       </c>
       <c r="J134" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K134" t="str">
         <v>9175550100</v>
       </c>
       <c r="L134" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M134" t="str">
         <v>6465550100</v>
       </c>
       <c r="N134" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O134" t="str">
         <v/>
@@ -7932,19 +7932,19 @@
         <v>2125550100</v>
       </c>
       <c r="J135" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K135" t="str">
         <v>9175550100</v>
       </c>
       <c r="L135" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M135" t="str">
         <v>6465550100</v>
       </c>
       <c r="N135" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O135" t="str">
         <v/>
@@ -7988,19 +7988,19 @@
         <v>2125550100</v>
       </c>
       <c r="J136" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K136" t="str">
         <v>9175550100</v>
       </c>
       <c r="L136" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M136" t="str">
         <v>6465550100</v>
       </c>
       <c r="N136" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O136" t="str">
         <v/>
@@ -8044,19 +8044,19 @@
         <v>2125550100</v>
       </c>
       <c r="J137" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K137" t="str">
         <v>9175550100</v>
       </c>
       <c r="L137" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M137" t="str">
         <v>6465550100</v>
       </c>
       <c r="N137" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O137" t="str">
         <v/>
@@ -8100,19 +8100,19 @@
         <v>2125550100</v>
       </c>
       <c r="J138" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K138" t="str">
         <v>9175550100</v>
       </c>
       <c r="L138" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M138" t="str">
         <v>6465550100</v>
       </c>
       <c r="N138" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O138" t="str">
         <v/>
@@ -8156,19 +8156,19 @@
         <v>2125550100</v>
       </c>
       <c r="J139" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K139" t="str">
         <v>9175550100</v>
       </c>
       <c r="L139" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M139" t="str">
         <v>6465550100</v>
       </c>
       <c r="N139" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O139" t="str">
         <v/>
@@ -8212,19 +8212,19 @@
         <v>2125550100</v>
       </c>
       <c r="J140" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K140" t="str">
         <v>9175550100</v>
       </c>
       <c r="L140" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M140" t="str">
         <v>6465550100</v>
       </c>
       <c r="N140" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O140" t="str">
         <v/>
@@ -8268,19 +8268,19 @@
         <v>2125550100</v>
       </c>
       <c r="J141" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K141" t="str">
         <v>9175550100</v>
       </c>
       <c r="L141" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M141" t="str">
         <v>6465550100</v>
       </c>
       <c r="N141" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O141" t="str">
         <v/>
@@ -8324,19 +8324,19 @@
         <v>2125550100</v>
       </c>
       <c r="J142" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K142" t="str">
         <v>9175550100</v>
       </c>
       <c r="L142" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M142" t="str">
         <v>6465550100</v>
       </c>
       <c r="N142" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O142" t="str">
         <v/>
@@ -8380,19 +8380,19 @@
         <v>2125550100</v>
       </c>
       <c r="J143" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K143" t="str">
         <v>9175550100</v>
       </c>
       <c r="L143" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M143" t="str">
         <v>6465550100</v>
       </c>
       <c r="N143" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O143" t="str">
         <v/>
@@ -8436,19 +8436,19 @@
         <v>2125550100</v>
       </c>
       <c r="J144" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K144" t="str">
         <v>9175550100</v>
       </c>
       <c r="L144" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M144" t="str">
         <v>6465550100</v>
       </c>
       <c r="N144" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O144" t="str">
         <v/>
@@ -8492,19 +8492,19 @@
         <v>2125550100</v>
       </c>
       <c r="J145" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K145" t="str">
         <v>9175550100</v>
       </c>
       <c r="L145" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M145" t="str">
         <v>6465550100</v>
       </c>
       <c r="N145" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O145" t="str">
         <v/>
@@ -8548,19 +8548,19 @@
         <v>2125550100</v>
       </c>
       <c r="J146" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K146" t="str">
         <v>9175550100</v>
       </c>
       <c r="L146" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M146" t="str">
         <v>6465550100</v>
       </c>
       <c r="N146" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O146" t="str">
         <v/>
@@ -8604,19 +8604,19 @@
         <v>2125550100</v>
       </c>
       <c r="J147" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K147" t="str">
         <v>9175550100</v>
       </c>
       <c r="L147" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M147" t="str">
         <v>6465550100</v>
       </c>
       <c r="N147" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O147" t="str">
         <v/>
@@ -8660,19 +8660,19 @@
         <v>2125550100</v>
       </c>
       <c r="J148" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K148" t="str">
         <v>9175550100</v>
       </c>
       <c r="L148" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M148" t="str">
         <v>6465550100</v>
       </c>
       <c r="N148" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O148" t="str">
         <v/>
@@ -8716,19 +8716,19 @@
         <v>2125550100</v>
       </c>
       <c r="J149" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K149" t="str">
         <v>9175550100</v>
       </c>
       <c r="L149" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M149" t="str">
         <v>6465550100</v>
       </c>
       <c r="N149" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O149" t="str">
         <v/>
@@ -8772,19 +8772,19 @@
         <v>2125550100</v>
       </c>
       <c r="J150" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K150" t="str">
         <v>9175550100</v>
       </c>
       <c r="L150" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M150" t="str">
         <v>6465550100</v>
       </c>
       <c r="N150" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O150" t="str">
         <v/>
@@ -8828,19 +8828,19 @@
         <v>2125550100</v>
       </c>
       <c r="J151" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K151" t="str">
         <v>9175550100</v>
       </c>
       <c r="L151" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M151" t="str">
         <v>6465550100</v>
       </c>
       <c r="N151" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O151" t="str">
         <v/>
@@ -8884,19 +8884,19 @@
         <v>2125550100</v>
       </c>
       <c r="J152" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K152" t="str">
         <v>9175550100</v>
       </c>
       <c r="L152" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M152" t="str">
         <v>6465550100</v>
       </c>
       <c r="N152" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O152" t="str">
         <v/>
@@ -8940,19 +8940,19 @@
         <v>2125550100</v>
       </c>
       <c r="J153" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K153" t="str">
         <v>9175550100</v>
       </c>
       <c r="L153" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M153" t="str">
         <v>6465550100</v>
       </c>
       <c r="N153" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O153" t="str">
         <v/>
@@ -8996,19 +8996,19 @@
         <v>2125550100</v>
       </c>
       <c r="J154" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K154" t="str">
         <v>9175550100</v>
       </c>
       <c r="L154" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M154" t="str">
         <v>6465550100</v>
       </c>
       <c r="N154" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O154" t="str">
         <v/>
@@ -9052,19 +9052,19 @@
         <v>2125550100</v>
       </c>
       <c r="J155" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K155" t="str">
         <v>9175550100</v>
       </c>
       <c r="L155" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M155" t="str">
         <v>6465550100</v>
       </c>
       <c r="N155" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O155" t="str">
         <v/>
@@ -9108,19 +9108,19 @@
         <v>2125550100</v>
       </c>
       <c r="J156" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K156" t="str">
         <v>9175550100</v>
       </c>
       <c r="L156" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M156" t="str">
         <v>6465550100</v>
       </c>
       <c r="N156" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O156" t="str">
         <v/>
@@ -9164,19 +9164,19 @@
         <v>2125550100</v>
       </c>
       <c r="J157" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K157" t="str">
         <v>9175550100</v>
       </c>
       <c r="L157" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M157" t="str">
         <v>6465550100</v>
       </c>
       <c r="N157" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O157" t="str">
         <v/>
@@ -9220,19 +9220,19 @@
         <v>2125550100</v>
       </c>
       <c r="J158" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K158" t="str">
         <v>9175550100</v>
       </c>
       <c r="L158" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M158" t="str">
         <v>6465550100</v>
       </c>
       <c r="N158" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O158" t="str">
         <v/>
@@ -9276,19 +9276,19 @@
         <v>2125550100</v>
       </c>
       <c r="J159" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K159" t="str">
         <v>9175550100</v>
       </c>
       <c r="L159" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M159" t="str">
         <v>6465550100</v>
       </c>
       <c r="N159" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O159" t="str">
         <v/>
@@ -9332,19 +9332,19 @@
         <v>2125550100</v>
       </c>
       <c r="J160" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K160" t="str">
         <v>9175550100</v>
       </c>
       <c r="L160" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M160" t="str">
         <v>6465550100</v>
       </c>
       <c r="N160" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O160" t="str">
         <v/>
@@ -9388,19 +9388,19 @@
         <v>2125550100</v>
       </c>
       <c r="J161" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K161" t="str">
         <v>9175550100</v>
       </c>
       <c r="L161" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M161" t="str">
         <v>6465550100</v>
       </c>
       <c r="N161" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O161" t="str">
         <v/>
@@ -9444,19 +9444,19 @@
         <v>2125550100</v>
       </c>
       <c r="J162" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K162" t="str">
         <v>9175550100</v>
       </c>
       <c r="L162" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M162" t="str">
         <v>6465550100</v>
       </c>
       <c r="N162" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O162" t="str">
         <v/>
@@ -9500,19 +9500,19 @@
         <v>2125550100</v>
       </c>
       <c r="J163" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K163" t="str">
         <v>9175550100</v>
       </c>
       <c r="L163" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M163" t="str">
         <v>6465550100</v>
       </c>
       <c r="N163" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O163" t="str">
         <v/>
@@ -9556,19 +9556,19 @@
         <v>2125550100</v>
       </c>
       <c r="J164" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K164" t="str">
         <v>9175550100</v>
       </c>
       <c r="L164" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M164" t="str">
         <v>6465550100</v>
       </c>
       <c r="N164" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O164" t="str">
         <v/>
@@ -9612,19 +9612,19 @@
         <v>2125550100</v>
       </c>
       <c r="J165" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K165" t="str">
         <v>9175550100</v>
       </c>
       <c r="L165" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M165" t="str">
         <v>6465550100</v>
       </c>
       <c r="N165" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O165" t="str">
         <v/>
@@ -9668,19 +9668,19 @@
         <v>2125550100</v>
       </c>
       <c r="J166" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K166" t="str">
         <v>9175550100</v>
       </c>
       <c r="L166" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M166" t="str">
         <v>6465550100</v>
       </c>
       <c r="N166" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O166" t="str">
         <v/>
@@ -9724,19 +9724,19 @@
         <v>2125550100</v>
       </c>
       <c r="J167" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K167" t="str">
         <v>9175550100</v>
       </c>
       <c r="L167" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M167" t="str">
         <v>6465550100</v>
       </c>
       <c r="N167" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O167" t="str">
         <v/>
@@ -9780,19 +9780,19 @@
         <v>2125550100</v>
       </c>
       <c r="J168" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K168" t="str">
         <v>9175550100</v>
       </c>
       <c r="L168" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M168" t="str">
         <v>6465550100</v>
       </c>
       <c r="N168" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O168" t="str">
         <v/>
@@ -9836,19 +9836,19 @@
         <v>2125550100</v>
       </c>
       <c r="J169" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K169" t="str">
         <v>9175550100</v>
       </c>
       <c r="L169" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M169" t="str">
         <v>6465550100</v>
       </c>
       <c r="N169" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O169" t="str">
         <v/>
@@ -9892,19 +9892,19 @@
         <v>2125550100</v>
       </c>
       <c r="J170" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K170" t="str">
         <v>9175550100</v>
       </c>
       <c r="L170" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M170" t="str">
         <v>6465550100</v>
       </c>
       <c r="N170" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O170" t="str">
         <v/>
@@ -9948,19 +9948,19 @@
         <v>2125550100</v>
       </c>
       <c r="J171" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K171" t="str">
         <v>9175550100</v>
       </c>
       <c r="L171" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M171" t="str">
         <v>6465550100</v>
       </c>
       <c r="N171" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O171" t="str">
         <v/>
@@ -10004,19 +10004,19 @@
         <v>2125550100</v>
       </c>
       <c r="J172" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K172" t="str">
         <v>9175550100</v>
       </c>
       <c r="L172" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M172" t="str">
         <v>6465550100</v>
       </c>
       <c r="N172" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O172" t="str">
         <v/>
@@ -10060,19 +10060,19 @@
         <v>2125550100</v>
       </c>
       <c r="J173" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K173" t="str">
         <v>9175550100</v>
       </c>
       <c r="L173" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M173" t="str">
         <v>6465550100</v>
       </c>
       <c r="N173" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O173" t="str">
         <v/>
@@ -10116,19 +10116,19 @@
         <v>2125550100</v>
       </c>
       <c r="J174" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K174" t="str">
         <v>9175550100</v>
       </c>
       <c r="L174" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M174" t="str">
         <v>6465550100</v>
       </c>
       <c r="N174" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O174" t="str">
         <v/>
@@ -10172,19 +10172,19 @@
         <v>2125550100</v>
       </c>
       <c r="J175" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K175" t="str">
         <v>9175550100</v>
       </c>
       <c r="L175" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M175" t="str">
         <v>6465550100</v>
       </c>
       <c r="N175" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O175" t="str">
         <v/>
@@ -10228,19 +10228,19 @@
         <v>2125550100</v>
       </c>
       <c r="J176" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K176" t="str">
         <v>9175550100</v>
       </c>
       <c r="L176" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M176" t="str">
         <v>6465550100</v>
       </c>
       <c r="N176" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O176" t="str">
         <v/>
@@ -10284,19 +10284,19 @@
         <v>2125550100</v>
       </c>
       <c r="J177" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K177" t="str">
         <v>9175550100</v>
       </c>
       <c r="L177" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M177" t="str">
         <v>6465550100</v>
       </c>
       <c r="N177" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O177" t="str">
         <v/>
@@ -10340,19 +10340,19 @@
         <v>2125550100</v>
       </c>
       <c r="J178" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K178" t="str">
         <v>9175550100</v>
       </c>
       <c r="L178" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M178" t="str">
         <v>6465550100</v>
       </c>
       <c r="N178" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O178" t="str">
         <v/>
@@ -10396,19 +10396,19 @@
         <v>2125550100</v>
       </c>
       <c r="J179" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K179" t="str">
         <v>9175550100</v>
       </c>
       <c r="L179" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M179" t="str">
         <v>6465550100</v>
       </c>
       <c r="N179" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O179" t="str">
         <v/>
@@ -10452,19 +10452,19 @@
         <v>2125550100</v>
       </c>
       <c r="J180" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K180" t="str">
         <v>9175550100</v>
       </c>
       <c r="L180" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M180" t="str">
         <v>6465550100</v>
       </c>
       <c r="N180" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O180" t="str">
         <v/>
@@ -10508,19 +10508,19 @@
         <v>2125550100</v>
       </c>
       <c r="J181" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K181" t="str">
         <v>9175550100</v>
       </c>
       <c r="L181" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M181" t="str">
         <v>6465550100</v>
       </c>
       <c r="N181" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O181" t="str">
         <v/>
@@ -10564,19 +10564,19 @@
         <v>2125550100</v>
       </c>
       <c r="J182" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K182" t="str">
         <v>9175550100</v>
       </c>
       <c r="L182" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M182" t="str">
         <v>6465550100</v>
       </c>
       <c r="N182" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O182" t="str">
         <v/>
@@ -10620,19 +10620,19 @@
         <v>2125550100</v>
       </c>
       <c r="J183" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K183" t="str">
         <v>9175550100</v>
       </c>
       <c r="L183" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M183" t="str">
         <v>6465550100</v>
       </c>
       <c r="N183" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O183" t="str">
         <v/>
@@ -10676,19 +10676,19 @@
         <v>2125550100</v>
       </c>
       <c r="J184" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K184" t="str">
         <v>9175550100</v>
       </c>
       <c r="L184" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M184" t="str">
         <v>6465550100</v>
       </c>
       <c r="N184" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O184" t="str">
         <v/>
@@ -10732,19 +10732,19 @@
         <v>2125550100</v>
       </c>
       <c r="J185" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K185" t="str">
         <v>9175550100</v>
       </c>
       <c r="L185" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M185" t="str">
         <v>6465550100</v>
       </c>
       <c r="N185" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O185" t="str">
         <v/>
@@ -10788,19 +10788,19 @@
         <v>2125550100</v>
       </c>
       <c r="J186" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K186" t="str">
         <v>9175550100</v>
       </c>
       <c r="L186" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M186" t="str">
         <v>6465550100</v>
       </c>
       <c r="N186" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O186" t="str">
         <v/>
@@ -10844,19 +10844,19 @@
         <v>2125550100</v>
       </c>
       <c r="J187" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K187" t="str">
         <v>9175550100</v>
       </c>
       <c r="L187" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M187" t="str">
         <v>6465550100</v>
       </c>
       <c r="N187" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O187" t="str">
         <v/>
@@ -10900,19 +10900,19 @@
         <v>2125550100</v>
       </c>
       <c r="J188" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K188" t="str">
         <v>9175550100</v>
       </c>
       <c r="L188" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M188" t="str">
         <v>6465550100</v>
       </c>
       <c r="N188" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O188" t="str">
         <v/>
@@ -10956,19 +10956,19 @@
         <v>2125550100</v>
       </c>
       <c r="J189" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K189" t="str">
         <v>9175550100</v>
       </c>
       <c r="L189" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M189" t="str">
         <v>6465550100</v>
       </c>
       <c r="N189" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O189" t="str">
         <v/>
@@ -11012,19 +11012,19 @@
         <v>2125550100</v>
       </c>
       <c r="J190" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K190" t="str">
         <v>9175550100</v>
       </c>
       <c r="L190" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M190" t="str">
         <v>6465550100</v>
       </c>
       <c r="N190" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O190" t="str">
         <v/>
@@ -11068,19 +11068,19 @@
         <v>2125550100</v>
       </c>
       <c r="J191" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K191" t="str">
         <v>9175550100</v>
       </c>
       <c r="L191" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M191" t="str">
         <v>6465550100</v>
       </c>
       <c r="N191" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O191" t="str">
         <v/>
@@ -11124,19 +11124,19 @@
         <v>2125550100</v>
       </c>
       <c r="J192" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K192" t="str">
         <v>9175550100</v>
       </c>
       <c r="L192" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M192" t="str">
         <v>6465550100</v>
       </c>
       <c r="N192" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O192" t="str">
         <v/>
@@ -11180,19 +11180,19 @@
         <v>2125550100</v>
       </c>
       <c r="J193" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K193" t="str">
         <v>9175550100</v>
       </c>
       <c r="L193" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M193" t="str">
         <v>6465550100</v>
       </c>
       <c r="N193" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O193" t="str">
         <v/>
@@ -11236,19 +11236,19 @@
         <v>2125550100</v>
       </c>
       <c r="J194" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K194" t="str">
         <v>9175550100</v>
       </c>
       <c r="L194" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M194" t="str">
         <v>6465550100</v>
       </c>
       <c r="N194" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O194" t="str">
         <v/>
@@ -11292,19 +11292,19 @@
         <v>2125550100</v>
       </c>
       <c r="J195" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K195" t="str">
         <v>9175550100</v>
       </c>
       <c r="L195" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M195" t="str">
         <v>6465550100</v>
       </c>
       <c r="N195" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O195" t="str">
         <v/>
@@ -11348,19 +11348,19 @@
         <v>2125550100</v>
       </c>
       <c r="J196" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K196" t="str">
         <v>9175550100</v>
       </c>
       <c r="L196" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M196" t="str">
         <v>6465550100</v>
       </c>
       <c r="N196" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O196" t="str">
         <v/>
@@ -11404,19 +11404,19 @@
         <v>2125550100</v>
       </c>
       <c r="J197" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K197" t="str">
         <v>9175550100</v>
       </c>
       <c r="L197" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M197" t="str">
         <v>6465550100</v>
       </c>
       <c r="N197" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O197" t="str">
         <v/>
@@ -11460,19 +11460,19 @@
         <v>2125550100</v>
       </c>
       <c r="J198" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K198" t="str">
         <v>9175550100</v>
       </c>
       <c r="L198" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M198" t="str">
         <v>6465550100</v>
       </c>
       <c r="N198" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O198" t="str">
         <v/>
@@ -11516,19 +11516,19 @@
         <v>2125550100</v>
       </c>
       <c r="J199" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K199" t="str">
         <v>9175550100</v>
       </c>
       <c r="L199" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M199" t="str">
         <v>6465550100</v>
       </c>
       <c r="N199" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O199" t="str">
         <v/>
@@ -11572,19 +11572,19 @@
         <v>2125550100</v>
       </c>
       <c r="J200" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K200" t="str">
         <v>9175550100</v>
       </c>
       <c r="L200" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M200" t="str">
         <v>6465550100</v>
       </c>
       <c r="N200" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O200" t="str">
         <v/>
@@ -11628,19 +11628,19 @@
         <v>2125550100</v>
       </c>
       <c r="J201" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="K201" t="str">
         <v>9175550100</v>
       </c>
       <c r="L201" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="M201" t="str">
         <v>6465550100</v>
       </c>
       <c r="N201" t="str">
-        <v>1</v>
+        <v>United States(+1)</v>
       </c>
       <c r="O201" t="str">
         <v/>

</xml_diff>